<commit_message>
Fix Securitization: WAL was described, never actually computed
The tab is literally named "WAL & CPR" and had a 6-month sample paydown
schedule, but the WAL cell itself just said "compute once full schedule
is built" -- the one thing the tab promises in its own name was never
implemented.

Added the real formula: WAL (years) = sum(month x principal paid that
month) / total principal / 12, using SUMPRODUCT over the existing
scheduled-principal and prepayment columns.

Verified against an independent Python recomputation of the same
definition using the recalculated cash flows (not a parallel hand-derived
formula that could drift): $1M pool, 8% CPR, $1,000/mo scheduled principal
-> WAL 0.28998 years, matched the cross-check to 10 decimal places.

19_Structured_Finance_Securitization: 30 -> 32 formulas.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HRsbvuXZcdzPw9SqPDRRxr
</commit_message>
<xml_diff>
--- a/14_Options_Derivatives/_template_OPTIONS.xlsx
+++ b/14_Options_Derivatives/_template_OPTIONS.xlsx
@@ -352,80 +352,84 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -684,54 +688,54 @@
   <dimension ref="B2:C8"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="4"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="4" t="s">
         <v>9</v>
       </c>
     </row>
@@ -754,136 +758,136 @@
   <dimension ref="B2:F14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="16"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="5" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="C5" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="8" t="n">
+      <c r="F5" s="9" t="n">
         <f aca="false">(LN(C5/C6)+(C8-C9+0.5*C10^2)*C7)/(C10*SQRT(C7))</f>
         <v>0.15</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="F6" s="8" t="n">
+      <c r="F6" s="9" t="n">
         <f aca="false">F5-C10*SQRT(C7)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="10" t="n">
         <v>0.25</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="8" t="n">
+      <c r="F7" s="9" t="n">
         <f aca="false">NORMSDIST(F5)</f>
         <v>0.559617692370243</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="10" t="n">
+      <c r="C8" s="11" t="n">
         <v>0.045</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="F8" s="8" t="n">
+      <c r="F8" s="9" t="n">
         <f aca="false">NORMSDIST(F6)</f>
         <v>0.5</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="10" t="n">
+      <c r="C9" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="F9" s="8" t="n">
+      <c r="F9" s="9" t="n">
         <f aca="false">NORMSDIST(-F5)</f>
         <v>0.440382307629758</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="11" t="n">
+      <c r="C10" s="12" t="n">
         <v>0.3</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="F10" s="8" t="n">
+      <c r="F10" s="9" t="n">
         <f aca="false">NORMSDIST(-F6)</f>
         <v>0.5</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="5" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="12" t="n">
+      <c r="C13" s="13" t="n">
         <f aca="false">C5*EXP(-C9*C7)*F7-C6*EXP(-C8*C7)*F8</f>
         <v>6.5211170064626</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C14" s="12" t="n">
+      <c r="C14" s="13" t="n">
         <f aca="false">C6*EXP(-C8*C7)*F10-C5*EXP(-C9*C7)*F9</f>
         <v>5.4024214675859</v>
       </c>
@@ -907,109 +911,109 @@
   <dimension ref="A2:E9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="40"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13"/>
-      <c r="B4" s="13" t="s">
+      <c r="A4" s="14"/>
+      <c r="B4" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="8" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C5" s="8" t="n">
+      <c r="C5" s="9" t="n">
         <f aca="false">EXP(-'BS Pricer'!$C$9*'BS Pricer'!$C$7)*'BS Pricer'!$F$7</f>
         <v>0.559617692370243</v>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D5" s="9" t="n">
         <f aca="false">-EXP(-'BS Pricer'!$C$9*'BS Pricer'!$C$7)*'BS Pricer'!$F$9</f>
         <v>-0.440382307629758</v>
       </c>
-      <c r="E5" s="14" t="s">
+      <c r="E5" s="15" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="C6" s="8" t="n">
+      <c r="C6" s="9" t="n">
         <f aca="false">EXP(-'BS Pricer'!$C$9*'BS Pricer'!$C$7)*(EXP(-('BS Pricer'!$F$5)^2/2)/SQRT(2*PI()))/('BS Pricer'!$C$5*'BS Pricer'!$C$10*SQRT('BS Pricer'!$C$7))</f>
         <v>0.026897048103991</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="9" t="n">
         <f aca="false">EXP(-'BS Pricer'!$C$9*'BS Pricer'!$C$7)*(EXP(-('BS Pricer'!$F$5)^2/2)/SQRT(2*PI()))/('BS Pricer'!$C$5*'BS Pricer'!$C$10*SQRT('BS Pricer'!$C$7))</f>
         <v>0.026897048103991</v>
       </c>
-      <c r="E6" s="14" t="s">
+      <c r="E6" s="15" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="8" t="n">
+      <c r="C7" s="9" t="n">
         <f aca="false">'BS Pricer'!$C$5*EXP(-'BS Pricer'!$C$9*'BS Pricer'!$C$7)*(EXP(-('BS Pricer'!$F$5)^2/2)/SQRT(2*PI()))*SQRT('BS Pricer'!$C$7)/100</f>
         <v>0.201727860779933</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="9" t="n">
         <f aca="false">'BS Pricer'!$C$5*EXP(-'BS Pricer'!$C$9*'BS Pricer'!$C$7)*(EXP(-('BS Pricer'!$F$5)^2/2)/SQRT(2*PI()))*SQRT('BS Pricer'!$C$7)/100</f>
         <v>0.201727860779933</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E7" s="15" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="C8" s="9" t="n">
         <f aca="false">(-'BS Pricer'!$C$5*(EXP(-('BS Pricer'!$F$5)^2/2)/SQRT(2*PI()))*'BS Pricer'!$C$10*EXP(-'BS Pricer'!$C$9*'BS Pricer'!$C$7)/(2*SQRT('BS Pricer'!$C$7))-'BS Pricer'!$C$8*'BS Pricer'!$C$6*EXP(-'BS Pricer'!$C$8*'BS Pricer'!$C$7)*'BS Pricer'!$F$8+'BS Pricer'!$C$9*'BS Pricer'!$C$5*EXP(-'BS Pricer'!$C$9*'BS Pricer'!$C$7)*'BS Pricer'!$F$7)/365</f>
         <v>-0.0392561671155377</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="9" t="n">
         <f aca="false">(-'BS Pricer'!$C$5*(EXP(-('BS Pricer'!$F$5)^2/2)/SQRT(2*PI()))*'BS Pricer'!$C$10*EXP(-'BS Pricer'!$C$9*'BS Pricer'!$C$7)/(2*SQRT('BS Pricer'!$C$7))+'BS Pricer'!$C$8*'BS Pricer'!$C$6*EXP(-'BS Pricer'!$C$8*'BS Pricer'!$C$7)*'BS Pricer'!$F$10-'BS Pricer'!$C$9*'BS Pricer'!$C$5*EXP(-'BS Pricer'!$C$9*'BS Pricer'!$C$7)*'BS Pricer'!$F$9)/365</f>
         <v>-0.0270653213600567</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="15" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C9" s="8" t="n">
+      <c r="C9" s="9" t="n">
         <f aca="false">'BS Pricer'!$C$6*'BS Pricer'!$C$7*EXP(-'BS Pricer'!$C$8*'BS Pricer'!$C$7)*'BS Pricer'!$F$8/100</f>
         <v>0.123601630576404</v>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="9" t="n">
         <f aca="false">-'BS Pricer'!$C$6*'BS Pricer'!$C$7*EXP(-'BS Pricer'!$C$8*'BS Pricer'!$C$7)*'BS Pricer'!$F$10/100</f>
         <v>-0.123601630576404</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="E9" s="15" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1032,219 +1036,219 @@
   <dimension ref="B2:K11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="3" style="1" width="12"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C4" s="15" t="n">
+      <c r="C4" s="16" t="n">
         <v>70</v>
       </c>
-      <c r="D4" s="15" t="n">
+      <c r="D4" s="16" t="n">
         <v>80</v>
       </c>
-      <c r="E4" s="15" t="n">
+      <c r="E4" s="16" t="n">
         <v>90</v>
       </c>
-      <c r="F4" s="15" t="n">
+      <c r="F4" s="16" t="n">
         <v>100</v>
       </c>
-      <c r="G4" s="15" t="n">
+      <c r="G4" s="16" t="n">
         <v>110</v>
       </c>
-      <c r="H4" s="15" t="n">
+      <c r="H4" s="16" t="n">
         <v>120</v>
       </c>
-      <c r="I4" s="15" t="n">
+      <c r="I4" s="16" t="n">
         <v>130</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="16" t="n">
+      <c r="C5" s="17" t="n">
         <f aca="false">MAX(C4-'BS Pricer'!$C$6,0)</f>
         <v>0</v>
       </c>
-      <c r="D5" s="16" t="n">
+      <c r="D5" s="17" t="n">
         <f aca="false">MAX(D4-'BS Pricer'!$C$6,0)</f>
         <v>0</v>
       </c>
-      <c r="E5" s="16" t="n">
+      <c r="E5" s="17" t="n">
         <f aca="false">MAX(E4-'BS Pricer'!$C$6,0)</f>
         <v>0</v>
       </c>
-      <c r="F5" s="16" t="n">
+      <c r="F5" s="17" t="n">
         <f aca="false">MAX(F4-'BS Pricer'!$C$6,0)</f>
         <v>0</v>
       </c>
-      <c r="G5" s="16" t="n">
+      <c r="G5" s="17" t="n">
         <f aca="false">MAX(G4-'BS Pricer'!$C$6,0)</f>
         <v>10</v>
       </c>
-      <c r="H5" s="16" t="n">
+      <c r="H5" s="17" t="n">
         <f aca="false">MAX(H4-'BS Pricer'!$C$6,0)</f>
         <v>20</v>
       </c>
-      <c r="I5" s="16" t="n">
+      <c r="I5" s="17" t="n">
         <f aca="false">MAX(I4-'BS Pricer'!$C$6,0)</f>
         <v>30</v>
       </c>
-      <c r="J5" s="17"/>
-      <c r="K5" s="17"/>
+      <c r="J5" s="18"/>
+      <c r="K5" s="18"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="16" t="n">
+      <c r="C6" s="17" t="n">
         <f aca="false">MAX('BS Pricer'!$C$6-C4,0)</f>
         <v>30</v>
       </c>
-      <c r="D6" s="16" t="n">
+      <c r="D6" s="17" t="n">
         <f aca="false">MAX('BS Pricer'!$C$6-D4,0)</f>
         <v>20</v>
       </c>
-      <c r="E6" s="16" t="n">
+      <c r="E6" s="17" t="n">
         <f aca="false">MAX('BS Pricer'!$C$6-E4,0)</f>
         <v>10</v>
       </c>
-      <c r="F6" s="16" t="n">
+      <c r="F6" s="17" t="n">
         <f aca="false">MAX('BS Pricer'!$C$6-F4,0)</f>
         <v>0</v>
       </c>
-      <c r="G6" s="16" t="n">
+      <c r="G6" s="17" t="n">
         <f aca="false">MAX('BS Pricer'!$C$6-G4,0)</f>
         <v>0</v>
       </c>
-      <c r="H6" s="16" t="n">
+      <c r="H6" s="17" t="n">
         <f aca="false">MAX('BS Pricer'!$C$6-H4,0)</f>
         <v>0</v>
       </c>
-      <c r="I6" s="16" t="n">
+      <c r="I6" s="17" t="n">
         <f aca="false">MAX('BS Pricer'!$C$6-I4,0)</f>
         <v>0</v>
       </c>
-      <c r="J6" s="17"/>
-      <c r="K6" s="17"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="18"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="16" t="n">
+      <c r="C7" s="17" t="n">
         <f aca="false">C5+C6</f>
         <v>30</v>
       </c>
-      <c r="D7" s="16" t="n">
+      <c r="D7" s="17" t="n">
         <f aca="false">D5+D6</f>
         <v>20</v>
       </c>
-      <c r="E7" s="16" t="n">
+      <c r="E7" s="17" t="n">
         <f aca="false">E5+E6</f>
         <v>10</v>
       </c>
-      <c r="F7" s="16" t="n">
+      <c r="F7" s="17" t="n">
         <f aca="false">F5+F6</f>
         <v>0</v>
       </c>
-      <c r="G7" s="16" t="n">
+      <c r="G7" s="17" t="n">
         <f aca="false">G5+G6</f>
         <v>10</v>
       </c>
-      <c r="H7" s="16" t="n">
+      <c r="H7" s="17" t="n">
         <f aca="false">H5+H6</f>
         <v>20</v>
       </c>
-      <c r="I7" s="16" t="n">
+      <c r="I7" s="17" t="n">
         <f aca="false">I5+I6</f>
         <v>30</v>
       </c>
-      <c r="J7" s="17"/>
-      <c r="K7" s="17"/>
+      <c r="J7" s="18"/>
+      <c r="K7" s="18"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C8" s="16" t="n">
+      <c r="C8" s="17" t="n">
         <f aca="false">'BS Pricer'!$C$13+'BS Pricer'!$C$14</f>
         <v>11.9235384740485</v>
       </c>
-      <c r="D8" s="16" t="n">
+      <c r="D8" s="17" t="n">
         <f aca="false">'BS Pricer'!$C$13+'BS Pricer'!$C$14</f>
         <v>11.9235384740485</v>
       </c>
-      <c r="E8" s="16" t="n">
+      <c r="E8" s="17" t="n">
         <f aca="false">'BS Pricer'!$C$13+'BS Pricer'!$C$14</f>
         <v>11.9235384740485</v>
       </c>
-      <c r="F8" s="16" t="n">
+      <c r="F8" s="17" t="n">
         <f aca="false">'BS Pricer'!$C$13+'BS Pricer'!$C$14</f>
         <v>11.9235384740485</v>
       </c>
-      <c r="G8" s="16" t="n">
+      <c r="G8" s="17" t="n">
         <f aca="false">'BS Pricer'!$C$13+'BS Pricer'!$C$14</f>
         <v>11.9235384740485</v>
       </c>
-      <c r="H8" s="16" t="n">
+      <c r="H8" s="17" t="n">
         <f aca="false">'BS Pricer'!$C$13+'BS Pricer'!$C$14</f>
         <v>11.9235384740485</v>
       </c>
-      <c r="I8" s="16" t="n">
+      <c r="I8" s="17" t="n">
         <f aca="false">'BS Pricer'!$C$13+'BS Pricer'!$C$14</f>
         <v>11.9235384740485</v>
       </c>
-      <c r="J8" s="17"/>
-      <c r="K8" s="17"/>
+      <c r="J8" s="18"/>
+      <c r="K8" s="18"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="18" t="n">
+      <c r="C9" s="19" t="n">
         <f aca="false">C7-C8</f>
         <v>18.0764615259515</v>
       </c>
-      <c r="D9" s="18" t="n">
+      <c r="D9" s="19" t="n">
         <f aca="false">D7-D8</f>
         <v>8.0764615259515</v>
       </c>
-      <c r="E9" s="18" t="n">
+      <c r="E9" s="19" t="n">
         <f aca="false">E7-E8</f>
         <v>-1.9235384740485</v>
       </c>
-      <c r="F9" s="18" t="n">
+      <c r="F9" s="19" t="n">
         <f aca="false">F7-F8</f>
         <v>-11.9235384740485</v>
       </c>
-      <c r="G9" s="18" t="n">
+      <c r="G9" s="19" t="n">
         <f aca="false">G7-G8</f>
         <v>-1.9235384740485</v>
       </c>
-      <c r="H9" s="18" t="n">
+      <c r="H9" s="19" t="n">
         <f aca="false">H7-H8</f>
         <v>8.0764615259515</v>
       </c>
-      <c r="I9" s="18" t="n">
+      <c r="I9" s="19" t="n">
         <f aca="false">I7-I8</f>
         <v>18.0764615259515</v>
       </c>
-      <c r="J9" s="17"/>
-      <c r="K9" s="17"/>
+      <c r="J9" s="18"/>
+      <c r="K9" s="18"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="15" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1267,104 +1271,104 @@
   <dimension ref="B2:F14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="16"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="14" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="17"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
+      <c r="B5" s="18"/>
+      <c r="C5" s="18"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="17"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="17"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17"/>
+      <c r="B7" s="18"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="17"/>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
+      <c r="B8" s="18"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="17"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
+      <c r="B9" s="18"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="17"/>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="17"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
+      <c r="B11" s="18"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="18"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="18"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="17"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
+      <c r="B12" s="18"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="18"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="17"/>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
+      <c r="B13" s="18"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
+      <c r="E13" s="18"/>
+      <c r="F13" s="18"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="17"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
+      <c r="B14" s="18"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="18"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>